<commit_message>
Ware House and PR
</commit_message>
<xml_diff>
--- a/ZlaataQA/src/test/resources/testdata/zltUI/ZltTestData.xlsx
+++ b/ZlaataQA/src/test/resources/testdata/zltUI/ZltTestData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Abdul\git\AdminPanelV2new\ZlaataQA\src\test\resources\testdata\zltUI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sarojkumar\git\AdminPanelV233\ZlaataQA\src\test\resources\testdata\zltUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAB49758-839C-496C-91A7-0FD92E487233}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F710F0DC-FDD2-48FB-A35F-0BC37C1FFA2F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{905F911F-FA1A-4DDD-B945-7467E9458D34}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1039" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1272" uniqueCount="170">
   <si>
     <t>S.No</t>
   </si>
@@ -473,6 +473,69 @@
   </si>
   <si>
     <t>Verify that multiple raw materials can be added with available quantities and the calculated amount is displayed correctly</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_PR_01</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_PR_02</t>
+  </si>
+  <si>
+    <t>TD_UI_Zlaata_PR_01</t>
+  </si>
+  <si>
+    <t>TD_UI_Zlaata_PR_02</t>
+  </si>
+  <si>
+    <t>Verify that a newly created Purchase Receive In Transit Status is displayed on the Purchase Receive Listing page</t>
+  </si>
+  <si>
+    <t>Verify Purchase Receive the Received Status is displayed correctly on Listing and Preview Page.</t>
+  </si>
+  <si>
+    <t>Verify that the convert bill option should redirect to bill module.</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_PR_03</t>
+  </si>
+  <si>
+    <t>TD_UI_Zlaata_PR_03</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_PR_04</t>
+  </si>
+  <si>
+    <t>TD_UI_Zlaata_PR_04</t>
+  </si>
+  <si>
+    <t>Verify that validation messages are displayed when mandatory fields are left blank and the user tries to save the Purchase Receive</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_WH_01</t>
+  </si>
+  <si>
+    <t>Verify that a newly created WareHouse  is displayed on the WareHouse Listing page.</t>
+  </si>
+  <si>
+    <t>TD_UI_Zlaata_WH_01</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_WH_02</t>
+  </si>
+  <si>
+    <t>Verify that changes made after editing a WareHouse are updated correctly and displayed on the WareHouse Listing page.</t>
+  </si>
+  <si>
+    <t>TD_UI_Zlaata_WH_02</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_WH_03</t>
+  </si>
+  <si>
+    <t>TD_UI_Zlaata_WH_03</t>
+  </si>
+  <si>
+    <t>Verify that Set as main Branch functionalty.</t>
   </si>
 </sst>
 </file>
@@ -652,7 +715,127 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="54">
+  <dxfs count="66">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1509,7 +1692,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C75D1F84-2AD1-4552-9C1F-85B59D75CCFA}">
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
@@ -2599,8 +2782,262 @@
         <v>13</v>
       </c>
     </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A38" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="B38" s="15"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="15"/>
+      <c r="E38" s="15"/>
+      <c r="F38" s="15"/>
+      <c r="G38" s="15"/>
+      <c r="H38" s="15"/>
+      <c r="I38" s="15"/>
+      <c r="J38" s="15"/>
+    </row>
+    <row r="39" spans="1:10" s="13" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A39" s="13">
+        <v>1</v>
+      </c>
+      <c r="B39" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="D39" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="E39" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F39" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="G39" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H39" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="I39" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="J39" s="13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" s="13" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A40" s="13">
+        <v>2</v>
+      </c>
+      <c r="B40" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C40" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="D40" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="E40" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="G40" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H40" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="I40" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="J40" s="13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" s="13" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A41" s="13">
+        <v>3</v>
+      </c>
+      <c r="B41" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C41" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="D41" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="E41" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F41" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="G41" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H41" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="I41" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="J41" s="13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" s="13" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A42" s="13">
+        <v>4</v>
+      </c>
+      <c r="B42" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C42" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="D42" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="E42" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="G42" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H42" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="I42" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="J42" s="13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A43" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="B43" s="15"/>
+      <c r="C43" s="15"/>
+      <c r="D43" s="15"/>
+      <c r="E43" s="15"/>
+      <c r="F43" s="15"/>
+      <c r="G43" s="15"/>
+      <c r="H43" s="15"/>
+      <c r="I43" s="15"/>
+      <c r="J43" s="15"/>
+    </row>
+    <row r="44" spans="1:10" s="13" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A44" s="13">
+        <v>1</v>
+      </c>
+      <c r="B44" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D44" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="E44" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="G44" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H44" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="I44" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="J44" s="13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" s="13" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A45" s="13">
+        <v>2</v>
+      </c>
+      <c r="B45" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C45" s="13" t="s">
+        <v>164</v>
+      </c>
+      <c r="D45" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="E45" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="G45" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H45" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="I45" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="J45" s="13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" s="13" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A46" s="13">
+        <v>3</v>
+      </c>
+      <c r="B46" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C46" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="D46" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="E46" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="G46" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H46" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="I46" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="J46" s="13" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
+    <mergeCell ref="A43:J43"/>
+    <mergeCell ref="A38:J38"/>
     <mergeCell ref="A31:J31"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A9:J9"/>
@@ -2616,7 +3053,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE74813B-34A6-48F5-8B35-1C10409ED694}">
-  <dimension ref="A1:AG31"/>
+  <dimension ref="A1:AG38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="48.88671875" customWidth="1"/>
@@ -5236,214 +5673,851 @@
       <c r="AF31" s="3"/>
       <c r="AG31" s="3"/>
     </row>
+    <row r="32" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A32" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L32" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="P32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="R32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="S32" s="3"/>
+      <c r="T32" s="3"/>
+      <c r="U32" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="V32" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="W32" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="X32" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y32" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z32" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA32" s="3"/>
+      <c r="AB32" s="3"/>
+      <c r="AC32" s="3"/>
+      <c r="AD32" s="3"/>
+      <c r="AE32" s="3"/>
+      <c r="AF32" s="3"/>
+      <c r="AG32" s="3"/>
+    </row>
+    <row r="33" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A33" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L33" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="P33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="R33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="S33" s="3"/>
+      <c r="T33" s="3"/>
+      <c r="U33" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="V33" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="W33" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="X33" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y33" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z33" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA33" s="3"/>
+      <c r="AB33" s="3"/>
+      <c r="AC33" s="3"/>
+      <c r="AD33" s="3"/>
+      <c r="AE33" s="3"/>
+      <c r="AF33" s="3"/>
+      <c r="AG33" s="3"/>
+    </row>
+    <row r="34" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A34" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L34" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="P34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="R34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="S34" s="3"/>
+      <c r="T34" s="3"/>
+      <c r="U34" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="V34" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="W34" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="X34" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y34" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z34" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA34" s="3"/>
+      <c r="AB34" s="3"/>
+      <c r="AC34" s="3"/>
+      <c r="AD34" s="3"/>
+      <c r="AE34" s="3"/>
+      <c r="AF34" s="3"/>
+      <c r="AG34" s="3"/>
+    </row>
+    <row r="35" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A35" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L35" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="P35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="R35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="S35" s="3"/>
+      <c r="T35" s="3"/>
+      <c r="U35" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="V35" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="W35" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="X35" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y35" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z35" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA35" s="3"/>
+      <c r="AB35" s="3"/>
+      <c r="AC35" s="3"/>
+      <c r="AD35" s="3"/>
+      <c r="AE35" s="3"/>
+      <c r="AF35" s="3"/>
+      <c r="AG35" s="3"/>
+    </row>
+    <row r="36" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A36" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="K36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L36" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="P36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="R36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="S36" s="3"/>
+      <c r="T36" s="3"/>
+      <c r="U36" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="V36" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="W36" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="X36" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y36" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z36" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA36" s="3"/>
+      <c r="AB36" s="3"/>
+      <c r="AC36" s="3"/>
+      <c r="AD36" s="3"/>
+      <c r="AE36" s="3"/>
+      <c r="AF36" s="3"/>
+      <c r="AG36" s="3"/>
+    </row>
+    <row r="37" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A37" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L37" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="P37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="R37" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="S37" s="3"/>
+      <c r="T37" s="3"/>
+      <c r="U37" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="V37" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="W37" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="X37" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y37" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z37" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA37" s="3"/>
+      <c r="AB37" s="3"/>
+      <c r="AC37" s="3"/>
+      <c r="AD37" s="3"/>
+      <c r="AE37" s="3"/>
+      <c r="AF37" s="3"/>
+      <c r="AG37" s="3"/>
+    </row>
+    <row r="38" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A38" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="K38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L38" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="P38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="R38" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="S38" s="3"/>
+      <c r="T38" s="3"/>
+      <c r="U38" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="V38" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="W38" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="X38" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y38" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z38" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA38" s="3"/>
+      <c r="AB38" s="3"/>
+      <c r="AC38" s="3"/>
+      <c r="AD38" s="3"/>
+      <c r="AE38" s="3"/>
+      <c r="AF38" s="3"/>
+      <c r="AG38" s="3"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
   <conditionalFormatting sqref="A2">
-    <cfRule type="containsText" dxfId="53" priority="89" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="65" priority="103" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="52" priority="90" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="64" priority="104" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A8">
-    <cfRule type="containsText" dxfId="51" priority="63" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="63" priority="77" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A8)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="50" priority="64" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="62" priority="78" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A8)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A9">
-    <cfRule type="containsText" dxfId="49" priority="61" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="61" priority="75" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A9)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="48" priority="62" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="60" priority="76" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A9)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A10">
-    <cfRule type="containsText" dxfId="47" priority="59" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="59" priority="73" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A10)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="46" priority="60" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="58" priority="74" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A10)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3">
-    <cfRule type="containsText" dxfId="45" priority="57" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="57" priority="71" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="44" priority="58" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="56" priority="72" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A4">
-    <cfRule type="containsText" dxfId="43" priority="55" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="55" priority="69" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="42" priority="56" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="54" priority="70" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5">
-    <cfRule type="containsText" dxfId="41" priority="53" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="53" priority="67" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="40" priority="54" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="52" priority="68" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A11">
-    <cfRule type="containsText" dxfId="39" priority="51" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="51" priority="65" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="38" priority="52" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="50" priority="66" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A11)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A12">
-    <cfRule type="containsText" dxfId="37" priority="49" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="49" priority="63" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A12)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="36" priority="50" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="48" priority="64" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A12)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A13">
-    <cfRule type="containsText" dxfId="35" priority="47" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="47" priority="61" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A13)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="34" priority="48" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="46" priority="62" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A13)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A14">
-    <cfRule type="containsText" dxfId="33" priority="45" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="45" priority="59" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A14)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="32" priority="46" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="44" priority="60" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A14)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A15">
-    <cfRule type="containsText" dxfId="31" priority="43" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="43" priority="57" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A15)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="30" priority="44" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="42" priority="58" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A15)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A16">
-    <cfRule type="containsText" dxfId="29" priority="41" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="41" priority="55" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A16)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="28" priority="42" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="40" priority="56" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A16)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A17">
-    <cfRule type="containsText" dxfId="27" priority="39" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="39" priority="53" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A17)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="26" priority="40" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="38" priority="54" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A17)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A18">
-    <cfRule type="containsText" dxfId="25" priority="37" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="37" priority="51" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A18)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="24" priority="38" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="36" priority="52" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A18)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A19">
-    <cfRule type="containsText" dxfId="23" priority="35" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="35" priority="49" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A19)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="22" priority="36" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="34" priority="50" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A19)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A20">
-    <cfRule type="containsText" dxfId="21" priority="33" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="33" priority="47" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A20)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="20" priority="34" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="32" priority="48" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A20)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A21:A25">
-    <cfRule type="containsText" dxfId="19" priority="31" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="31" priority="45" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A21)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="18" priority="32" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="30" priority="46" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A21)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A6">
-    <cfRule type="containsText" dxfId="17" priority="17" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="29" priority="31" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="18" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="28" priority="32" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A6)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A7">
-    <cfRule type="containsText" dxfId="15" priority="15" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="27" priority="29" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A7)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="16" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="26" priority="30" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A7)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A26">
-    <cfRule type="containsText" dxfId="13" priority="13" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="25" priority="27" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A26)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="14" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="24" priority="28" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A26)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A27">
-    <cfRule type="containsText" dxfId="11" priority="11" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="23" priority="25" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A27)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="12" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="22" priority="26" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A27)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A28">
-    <cfRule type="containsText" dxfId="9" priority="9" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="21" priority="23" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A28)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="10" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="20" priority="24" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A28)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A29">
-    <cfRule type="containsText" dxfId="7" priority="7" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="19" priority="21" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A29)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="8" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="18" priority="22" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A29)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A30">
-    <cfRule type="containsText" dxfId="5" priority="5" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="17" priority="19" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A30)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="6" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="16" priority="20" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A30)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A31">
-    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="15" priority="17" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A31)))</formula>
     </cfRule>
+    <cfRule type="containsText" dxfId="14" priority="18" operator="containsText" text="&lt;EMPTY&gt;">
+      <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A31)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A32">
+    <cfRule type="containsText" dxfId="13" priority="13" operator="containsText" text="&lt;NA&gt;">
+      <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A32)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="12" priority="14" operator="containsText" text="&lt;EMPTY&gt;">
+      <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A32)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A33">
+    <cfRule type="containsText" dxfId="11" priority="11" operator="containsText" text="&lt;NA&gt;">
+      <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A33)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="10" priority="12" operator="containsText" text="&lt;EMPTY&gt;">
+      <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A33)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A34">
+    <cfRule type="containsText" dxfId="9" priority="9" operator="containsText" text="&lt;NA&gt;">
+      <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A34)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="8" priority="10" operator="containsText" text="&lt;EMPTY&gt;">
+      <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A34)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A35">
+    <cfRule type="containsText" dxfId="7" priority="7" operator="containsText" text="&lt;NA&gt;">
+      <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A35)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="6" priority="8" operator="containsText" text="&lt;EMPTY&gt;">
+      <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A35)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A36">
+    <cfRule type="containsText" dxfId="5" priority="5" operator="containsText" text="&lt;NA&gt;">
+      <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A36)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="6" operator="containsText" text="&lt;EMPTY&gt;">
+      <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A36)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A37">
+    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="&lt;NA&gt;">
+      <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A37)))</formula>
+    </cfRule>
     <cfRule type="containsText" dxfId="2" priority="4" operator="containsText" text="&lt;EMPTY&gt;">
-      <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A31)))</formula>
+      <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A37)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A38">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="&lt;NA&gt;">
+      <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A38)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="&lt;EMPTY&gt;">
+      <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A38)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Manufacture Order Automation Script.
</commit_message>
<xml_diff>
--- a/ZlaataQA/src/test/resources/testdata/zltUI/ZltTestData.xlsx
+++ b/ZlaataQA/src/test/resources/testdata/zltUI/ZltTestData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sarojkumar\git\AdminPanelV233\ZlaataQA\src\test\resources\testdata\zltUI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Abdul\git\AdminPanelV2Remote\ZlaataQA\src\test\resources\testdata\zltUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F710F0DC-FDD2-48FB-A35F-0BC37C1FFA2F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A07458E-0DDC-457C-BC96-D502E4BB58B9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{905F911F-FA1A-4DDD-B945-7467E9458D34}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1272" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1504" uniqueCount="194">
   <si>
     <t>S.No</t>
   </si>
@@ -536,6 +536,78 @@
   </si>
   <si>
     <t>Verify that Set as main Branch functionalty.</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_MO_01</t>
+  </si>
+  <si>
+    <t>Verify that a newly created Manufacture Order is displayed on the Manufacture Order Listing page</t>
+  </si>
+  <si>
+    <t>TD_UI_Zlaata_MO_01</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_MO_02</t>
+  </si>
+  <si>
+    <t>Verify that when a product is saved as Draft, the status is displayed as Draft and the Draft product can be deleted</t>
+  </si>
+  <si>
+    <t>TD_UI_Zlaata_MO_02</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_MO_03</t>
+  </si>
+  <si>
+    <t>Verify that the user is able to edit the Manufacture Order and the edited Manufacture Order details are reflected correctly</t>
+  </si>
+  <si>
+    <t>TD_UI_Zlaata_MO_03</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_MO_04</t>
+  </si>
+  <si>
+    <t>Verify that the "Cancel Items" option is available and that the order status changes to "Cancelled" after cancelling the items</t>
+  </si>
+  <si>
+    <t>TD_UI_Zlaata_MO_04</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_MO_05</t>
+  </si>
+  <si>
+    <t>Verify that when an Open Manufacture Order is marked as Issued, the status is changed to Issued on both the Listing page and Detail page</t>
+  </si>
+  <si>
+    <t>TD_UI_Zlaata_MO_05</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_MO_06</t>
+  </si>
+  <si>
+    <t>Verify that when the user tries to save a Manufacture Order without entering the mandatory details, the mandatory field validation messages are displayed</t>
+  </si>
+  <si>
+    <t>TD_UI_Zlaata_MO_06</t>
+  </si>
+  <si>
+    <t>TC_UI_Zlaata_MO_07</t>
+  </si>
+  <si>
+    <t>Verify that multiple products and raw materials can be added while creating a new Manufacture Order</t>
+  </si>
+  <si>
+    <t>TD_UI_Zlaata_MO_07</t>
+  </si>
+  <si>
+    <t>Manufacture Order</t>
+  </si>
+  <si>
+    <t>Warehouse</t>
+  </si>
+  <si>
+    <t>Purchase Receive</t>
   </si>
 </sst>
 </file>
@@ -715,7 +787,147 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="66">
+  <dxfs count="80">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1692,7 +1904,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C75D1F84-2AD1-4552-9C1F-85B59D75CCFA}">
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
@@ -2784,7 +2996,7 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="15" t="s">
-        <v>129</v>
+        <v>193</v>
       </c>
       <c r="B38" s="15"/>
       <c r="C38" s="15"/>
@@ -2926,7 +3138,7 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="15" t="s">
-        <v>129</v>
+        <v>192</v>
       </c>
       <c r="B43" s="15"/>
       <c r="C43" s="15"/>
@@ -3034,8 +3246,247 @@
         <v>13</v>
       </c>
     </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A47" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="B47" s="15"/>
+      <c r="C47" s="15"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="15"/>
+      <c r="F47" s="15"/>
+      <c r="G47" s="15"/>
+      <c r="H47" s="15"/>
+      <c r="I47" s="15"/>
+      <c r="J47" s="15"/>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>1</v>
+      </c>
+      <c r="B48" t="s">
+        <v>10</v>
+      </c>
+      <c r="C48" t="s">
+        <v>170</v>
+      </c>
+      <c r="D48" t="s">
+        <v>171</v>
+      </c>
+      <c r="E48" t="s">
+        <v>14</v>
+      </c>
+      <c r="F48" t="s">
+        <v>172</v>
+      </c>
+      <c r="G48" t="s">
+        <v>11</v>
+      </c>
+      <c r="H48" t="s">
+        <v>133</v>
+      </c>
+      <c r="I48" t="s">
+        <v>12</v>
+      </c>
+      <c r="J48" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>2</v>
+      </c>
+      <c r="B49" t="s">
+        <v>10</v>
+      </c>
+      <c r="C49" t="s">
+        <v>173</v>
+      </c>
+      <c r="D49" t="s">
+        <v>177</v>
+      </c>
+      <c r="E49" t="s">
+        <v>14</v>
+      </c>
+      <c r="F49" t="s">
+        <v>175</v>
+      </c>
+      <c r="G49" t="s">
+        <v>11</v>
+      </c>
+      <c r="H49" t="s">
+        <v>133</v>
+      </c>
+      <c r="I49" t="s">
+        <v>12</v>
+      </c>
+      <c r="J49" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>3</v>
+      </c>
+      <c r="B50" t="s">
+        <v>10</v>
+      </c>
+      <c r="C50" t="s">
+        <v>176</v>
+      </c>
+      <c r="D50" t="s">
+        <v>174</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50" t="s">
+        <v>178</v>
+      </c>
+      <c r="G50" t="s">
+        <v>11</v>
+      </c>
+      <c r="H50" t="s">
+        <v>133</v>
+      </c>
+      <c r="I50" t="s">
+        <v>12</v>
+      </c>
+      <c r="J50" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>4</v>
+      </c>
+      <c r="B51" t="s">
+        <v>10</v>
+      </c>
+      <c r="C51" t="s">
+        <v>179</v>
+      </c>
+      <c r="D51" t="s">
+        <v>180</v>
+      </c>
+      <c r="E51" t="s">
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>181</v>
+      </c>
+      <c r="G51" t="s">
+        <v>11</v>
+      </c>
+      <c r="H51" t="s">
+        <v>133</v>
+      </c>
+      <c r="I51" t="s">
+        <v>12</v>
+      </c>
+      <c r="J51" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>5</v>
+      </c>
+      <c r="B52" t="s">
+        <v>10</v>
+      </c>
+      <c r="C52" t="s">
+        <v>182</v>
+      </c>
+      <c r="D52" t="s">
+        <v>183</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52" t="s">
+        <v>184</v>
+      </c>
+      <c r="G52" t="s">
+        <v>11</v>
+      </c>
+      <c r="H52" t="s">
+        <v>133</v>
+      </c>
+      <c r="I52" t="s">
+        <v>12</v>
+      </c>
+      <c r="J52" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>6</v>
+      </c>
+      <c r="B53" t="s">
+        <v>10</v>
+      </c>
+      <c r="C53" t="s">
+        <v>185</v>
+      </c>
+      <c r="D53" t="s">
+        <v>186</v>
+      </c>
+      <c r="E53" t="s">
+        <v>14</v>
+      </c>
+      <c r="F53" t="s">
+        <v>187</v>
+      </c>
+      <c r="G53" t="s">
+        <v>11</v>
+      </c>
+      <c r="H53" t="s">
+        <v>133</v>
+      </c>
+      <c r="I53" t="s">
+        <v>12</v>
+      </c>
+      <c r="J53" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A54">
+        <v>7</v>
+      </c>
+      <c r="B54" t="s">
+        <v>10</v>
+      </c>
+      <c r="C54" t="s">
+        <v>188</v>
+      </c>
+      <c r="D54" t="s">
+        <v>189</v>
+      </c>
+      <c r="E54" t="s">
+        <v>14</v>
+      </c>
+      <c r="F54" t="s">
+        <v>190</v>
+      </c>
+      <c r="G54" t="s">
+        <v>11</v>
+      </c>
+      <c r="H54" t="s">
+        <v>133</v>
+      </c>
+      <c r="I54" t="s">
+        <v>12</v>
+      </c>
+      <c r="J54" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
+    <mergeCell ref="A47:J47"/>
     <mergeCell ref="A43:J43"/>
     <mergeCell ref="A38:J38"/>
     <mergeCell ref="A31:J31"/>
@@ -3053,7 +3504,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE74813B-34A6-48F5-8B35-1C10409ED694}">
-  <dimension ref="A1:AG38"/>
+  <dimension ref="A1:AG45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="48.88671875" customWidth="1"/>
@@ -6254,270 +6705,859 @@
       <c r="AF38" s="3"/>
       <c r="AG38" s="3"/>
     </row>
+    <row r="39" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A39" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="K39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L39" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="P39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="R39" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="S39" s="3"/>
+      <c r="T39" s="3"/>
+      <c r="U39" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="V39" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="W39" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="X39" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y39" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z39" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA39" s="3"/>
+      <c r="AB39" s="3"/>
+      <c r="AC39" s="3"/>
+      <c r="AD39" s="3"/>
+      <c r="AE39" s="3"/>
+      <c r="AF39" s="3"/>
+      <c r="AG39" s="3"/>
+    </row>
+    <row r="40" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A40" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G40" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I40" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J40" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="K40" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L40" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M40" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N40" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O40" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="P40" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q40" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="R40" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="S40" s="3"/>
+      <c r="T40" s="3"/>
+      <c r="U40" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="V40" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="W40" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="X40" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y40" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z40" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA40" s="3"/>
+      <c r="AB40" s="3"/>
+      <c r="AC40" s="3"/>
+      <c r="AD40" s="3"/>
+      <c r="AE40" s="3"/>
+      <c r="AF40" s="3"/>
+      <c r="AG40" s="3"/>
+    </row>
+    <row r="41" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A41" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I41" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J41" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="K41" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L41" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M41" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N41" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O41" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="P41" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q41" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="R41" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="S41" s="3"/>
+      <c r="T41" s="3"/>
+      <c r="U41" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="V41" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="W41" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="X41" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y41" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z41" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA41" s="3"/>
+      <c r="AB41" s="3"/>
+      <c r="AC41" s="3"/>
+      <c r="AD41" s="3"/>
+      <c r="AE41" s="3"/>
+      <c r="AF41" s="3"/>
+      <c r="AG41" s="3"/>
+    </row>
+    <row r="42" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A42" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G42" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H42" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I42" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J42" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="K42" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L42" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M42" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N42" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O42" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="P42" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q42" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="R42" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="S42" s="3"/>
+      <c r="T42" s="3"/>
+      <c r="U42" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="V42" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="W42" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="X42" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y42" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z42" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA42" s="3"/>
+      <c r="AB42" s="3"/>
+      <c r="AC42" s="3"/>
+      <c r="AD42" s="3"/>
+      <c r="AE42" s="3"/>
+      <c r="AF42" s="3"/>
+      <c r="AG42" s="3"/>
+    </row>
+    <row r="43" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A43" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G43" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H43" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I43" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J43" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="K43" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L43" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M43" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N43" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O43" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="P43" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q43" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="R43" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="S43" s="3"/>
+      <c r="T43" s="3"/>
+      <c r="U43" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="V43" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="W43" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="X43" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y43" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z43" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA43" s="3"/>
+      <c r="AB43" s="3"/>
+      <c r="AC43" s="3"/>
+      <c r="AD43" s="3"/>
+      <c r="AE43" s="3"/>
+      <c r="AF43" s="3"/>
+      <c r="AG43" s="3"/>
+    </row>
+    <row r="44" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A44" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F44" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G44" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H44" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I44" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J44" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="K44" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L44" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M44" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N44" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O44" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="P44" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q44" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="R44" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="S44" s="3"/>
+      <c r="T44" s="3"/>
+      <c r="U44" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="V44" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="W44" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="X44" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y44" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z44" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA44" s="3"/>
+      <c r="AB44" s="3"/>
+      <c r="AC44" s="3"/>
+      <c r="AD44" s="3"/>
+      <c r="AE44" s="3"/>
+      <c r="AF44" s="3"/>
+      <c r="AG44" s="3"/>
+    </row>
+    <row r="45" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A45" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E45" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F45" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I45" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J45" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="K45" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L45" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M45" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N45" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O45" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="P45" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q45" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="R45" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="S45" s="3"/>
+      <c r="T45" s="3"/>
+      <c r="U45" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="V45" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="W45" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="X45" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y45" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z45" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA45" s="3"/>
+      <c r="AB45" s="3"/>
+      <c r="AC45" s="3"/>
+      <c r="AD45" s="3"/>
+      <c r="AE45" s="3"/>
+      <c r="AF45" s="3"/>
+      <c r="AG45" s="3"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
   <conditionalFormatting sqref="A2">
-    <cfRule type="containsText" dxfId="65" priority="103" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="79" priority="117" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="64" priority="104" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="78" priority="118" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A8">
-    <cfRule type="containsText" dxfId="63" priority="77" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="77" priority="91" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A8)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="62" priority="78" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="76" priority="92" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A8)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A9">
-    <cfRule type="containsText" dxfId="61" priority="75" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="75" priority="89" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A9)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="60" priority="76" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="74" priority="90" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A9)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A10">
-    <cfRule type="containsText" dxfId="59" priority="73" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="73" priority="87" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A10)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="58" priority="74" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="72" priority="88" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A10)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3">
-    <cfRule type="containsText" dxfId="57" priority="71" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="71" priority="85" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="56" priority="72" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="70" priority="86" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A4">
-    <cfRule type="containsText" dxfId="55" priority="69" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="69" priority="83" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="54" priority="70" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="68" priority="84" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5">
-    <cfRule type="containsText" dxfId="53" priority="67" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="67" priority="81" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="52" priority="68" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="66" priority="82" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A11">
-    <cfRule type="containsText" dxfId="51" priority="65" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="65" priority="79" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="50" priority="66" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="64" priority="80" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A11)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A12">
-    <cfRule type="containsText" dxfId="49" priority="63" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="63" priority="77" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A12)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="48" priority="64" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="62" priority="78" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A12)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A13">
-    <cfRule type="containsText" dxfId="47" priority="61" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="61" priority="75" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A13)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="46" priority="62" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="60" priority="76" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A13)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A14">
-    <cfRule type="containsText" dxfId="45" priority="59" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="59" priority="73" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A14)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="44" priority="60" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="58" priority="74" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A14)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A15">
-    <cfRule type="containsText" dxfId="43" priority="57" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="57" priority="71" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A15)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="42" priority="58" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="56" priority="72" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A15)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A16">
-    <cfRule type="containsText" dxfId="41" priority="55" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="55" priority="69" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A16)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="40" priority="56" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="54" priority="70" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A16)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A17">
-    <cfRule type="containsText" dxfId="39" priority="53" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="53" priority="67" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A17)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="38" priority="54" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="52" priority="68" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A17)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A18">
-    <cfRule type="containsText" dxfId="37" priority="51" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="51" priority="65" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A18)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="36" priority="52" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="50" priority="66" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A18)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A19">
-    <cfRule type="containsText" dxfId="35" priority="49" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="49" priority="63" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A19)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="34" priority="50" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="48" priority="64" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A19)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A20">
-    <cfRule type="containsText" dxfId="33" priority="47" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="47" priority="61" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A20)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="32" priority="48" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="46" priority="62" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A20)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A21:A25">
-    <cfRule type="containsText" dxfId="31" priority="45" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="45" priority="59" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A21)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="30" priority="46" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="44" priority="60" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A21)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A6">
-    <cfRule type="containsText" dxfId="29" priority="31" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="43" priority="45" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="28" priority="32" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="42" priority="46" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A6)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A7">
-    <cfRule type="containsText" dxfId="27" priority="29" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="41" priority="43" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A7)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="26" priority="30" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="40" priority="44" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A7)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A26">
-    <cfRule type="containsText" dxfId="25" priority="27" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="39" priority="41" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A26)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="24" priority="28" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="38" priority="42" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A26)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A27">
-    <cfRule type="containsText" dxfId="23" priority="25" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="37" priority="39" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A27)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="22" priority="26" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="36" priority="40" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A27)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A28">
-    <cfRule type="containsText" dxfId="21" priority="23" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="35" priority="37" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A28)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="20" priority="24" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="34" priority="38" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A28)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A29">
-    <cfRule type="containsText" dxfId="19" priority="21" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="33" priority="35" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A29)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="18" priority="22" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="32" priority="36" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A29)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A30">
-    <cfRule type="containsText" dxfId="17" priority="19" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="31" priority="33" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A30)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="20" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="30" priority="34" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A30)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A31">
-    <cfRule type="containsText" dxfId="15" priority="17" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="29" priority="31" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A31)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="18" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="28" priority="32" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A31)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A32">
-    <cfRule type="containsText" dxfId="13" priority="13" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="27" priority="27" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A32)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="14" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="26" priority="28" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A32)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A33">
-    <cfRule type="containsText" dxfId="11" priority="11" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="25" priority="25" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A33)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="12" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="24" priority="26" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A33)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A34">
-    <cfRule type="containsText" dxfId="9" priority="9" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="23" priority="23" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A34)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="10" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="22" priority="24" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A34)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A35">
-    <cfRule type="containsText" dxfId="7" priority="7" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="21" priority="21" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A35)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="8" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="20" priority="22" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A35)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A36">
-    <cfRule type="containsText" dxfId="5" priority="5" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="19" priority="19" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A36)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="6" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="18" priority="20" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A36)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A37">
-    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="17" priority="17" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A37)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="4" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="16" priority="18" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A37)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A38">
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="&lt;NA&gt;">
+    <cfRule type="containsText" dxfId="15" priority="15" operator="containsText" text="&lt;NA&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A38)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="&lt;EMPTY&gt;">
+    <cfRule type="containsText" dxfId="14" priority="16" operator="containsText" text="&lt;EMPTY&gt;">
       <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A38)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A39:A45">
+    <cfRule type="containsText" dxfId="13" priority="13" operator="containsText" text="&lt;NA&gt;">
+      <formula>NOT(ISERROR(SEARCH("&lt;NA&gt;",A39)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="12" priority="14" operator="containsText" text="&lt;EMPTY&gt;">
+      <formula>NOT(ISERROR(SEARCH("&lt;EMPTY&gt;",A39)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>